<commit_message>
updated source files with FY24 data, and ran CSV script (updating csv files).  next todo: run report qmd
</commit_message>
<xml_diff>
--- a/bin/peer_review_source.xlsx
+++ b/bin/peer_review_source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa-report\bin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4BEAC9-FC30-4F0B-B26D-2DC106C08394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C3344A-F561-4B64-A055-1892E9DADB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="12" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="18" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
   </bookViews>
   <sheets>
     <sheet name="FY06" sheetId="15" r:id="rId1"/>
@@ -31,6 +31,7 @@
     <sheet name="FY21" sheetId="28" r:id="rId16"/>
     <sheet name="FY22" sheetId="29" r:id="rId17"/>
     <sheet name="FY23" sheetId="30" r:id="rId18"/>
+    <sheet name="FY24" sheetId="31" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="3" hidden="1">'FY09'!#REF!</definedName>
@@ -62,6 +63,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -137,7 +140,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="151">
   <si>
     <t>None</t>
   </si>
@@ -563,13 +566,46 @@
   <si>
     <t>National Toxicology Program
 Environmental Health Sciences</t>
+  </si>
+  <si>
+    <t>APHIS</t>
+  </si>
+  <si>
+    <t>NOAA</t>
+  </si>
+  <si>
+    <t>Grid Deployment Office</t>
+  </si>
+  <si>
+    <t>OCSPP</t>
+  </si>
+  <si>
+    <t>ORD</t>
+  </si>
+  <si>
+    <t>BLM</t>
+  </si>
+  <si>
+    <t>OSMRE</t>
+  </si>
+  <si>
+    <t>BIA</t>
+  </si>
+  <si>
+    <t>BIE</t>
+  </si>
+  <si>
+    <t>BFTA</t>
+  </si>
+  <si>
+    <t>Agency10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -582,6 +618,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -614,10 +656,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -626,9 +669,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal_FY24" xfId="1" xr:uid="{5D0706CB-5128-4252-B37D-B6524F79CB82}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -644,9 +690,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -684,7 +730,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -790,7 +836,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -932,7 +978,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4223,6 +4269,278 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{690A201D-3511-49E4-82E5-F19DAF3BA1E0}">
+  <dimension ref="A1:Q12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="43.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="26" style="4" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" style="4" customWidth="1"/>
+    <col min="4" max="5" width="32" style="4" customWidth="1"/>
+    <col min="6" max="6" width="37.85546875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="31.85546875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" style="4" customWidth="1"/>
+    <col min="9" max="10" width="9.140625" style="4"/>
+    <col min="11" max="11" width="11.85546875" style="4" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4">
+        <f t="shared" ref="E3:E12" si="0">SUM(C5:D5)</f>
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G6" s="4">
+        <v>2</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="4">
+        <v>9</v>
+      </c>
+      <c r="E9" s="4">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="6">
+        <v>194</v>
+      </c>
+      <c r="D11" s="6">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4">
+        <f t="shared" si="0"/>
+        <v>197</v>
+      </c>
+      <c r="F11" s="4">
+        <v>30</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12" s="4">
+        <v>16</v>
+      </c>
+      <c r="E12" s="4">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="https://www.usgs.gov/office-of-science-quality-and-integrity/fundamental-science-practices/information-quality-usgs-peer-review-agenda" xr:uid="{08BE9C63-F0DE-4A5F-BE9B-A36C8E39E741}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
cleaned-up agency names in post-FY19 peer review source files, re-ran csv script
</commit_message>
<xml_diff>
--- a/bin/peer_review_source.xlsx
+++ b/bin/peer_review_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C3344A-F561-4B64-A055-1892E9DADB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9457C3B5-DD71-42CA-A0E4-4208B86B6A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="18" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="17" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
   </bookViews>
   <sheets>
     <sheet name="FY06" sheetId="15" r:id="rId1"/>
@@ -140,7 +140,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="134">
   <si>
     <t>None</t>
   </si>
@@ -148,9 +148,6 @@
     <t>7 (Waiver)</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>Agency1</t>
   </si>
   <si>
@@ -305,9 +302,6 @@
   </si>
   <si>
     <t>Bureau of Safety and Environmental Enforcement</t>
-  </si>
-  <si>
-    <t>3</t>
   </si>
   <si>
     <t>1</t>
@@ -437,21 +431,9 @@
     <t>Reviews of ISI</t>
   </si>
   <si>
-    <t>BSEE</t>
-  </si>
-  <si>
-    <t>USGS</t>
-  </si>
-  <si>
-    <t>FS</t>
-  </si>
-  <si>
     <t>Reclamation</t>
   </si>
   <si>
-    <t>FWS</t>
-  </si>
-  <si>
     <t>Waivers, Deferrals, or Exemptions (ISI)</t>
   </si>
   <si>
@@ -467,15 +449,6 @@
     <t xml:space="preserve">Potential Reviewer Conflicts </t>
   </si>
   <si>
-    <t>BOEM</t>
-  </si>
-  <si>
-    <t>FSIS</t>
-  </si>
-  <si>
-    <t>USAID</t>
-  </si>
-  <si>
     <t>Department of State</t>
   </si>
   <si>
@@ -483,15 +456,6 @@
   </si>
   <si>
     <t>Consumer Financial Protection Bureau</t>
-  </si>
-  <si>
-    <t>CDC</t>
-  </si>
-  <si>
-    <t>NIH</t>
-  </si>
-  <si>
-    <t>FDA</t>
   </si>
   <si>
     <t>Agency (abbrv.)</t>
@@ -568,37 +532,22 @@
 Environmental Health Sciences</t>
   </si>
   <si>
-    <t>APHIS</t>
-  </si>
-  <si>
-    <t>NOAA</t>
-  </si>
-  <si>
     <t>Grid Deployment Office</t>
   </si>
   <si>
-    <t>OCSPP</t>
-  </si>
-  <si>
-    <t>ORD</t>
-  </si>
-  <si>
-    <t>BLM</t>
-  </si>
-  <si>
-    <t>OSMRE</t>
-  </si>
-  <si>
-    <t>BIA</t>
-  </si>
-  <si>
-    <t>BIE</t>
-  </si>
-  <si>
-    <t>BFTA</t>
-  </si>
-  <si>
     <t>Agency10</t>
+  </si>
+  <si>
+    <t>Food Safety and Inspection Service</t>
+  </si>
+  <si>
+    <t>United States Agency for International Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bureau of Safety and Environmental Enforcement </t>
+  </si>
+  <si>
+    <t>United States Geological Survey</t>
   </si>
 </sst>
 </file>
@@ -1001,48 +950,48 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>82</v>
       </c>
-      <c r="G1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H1" t="s">
-        <v>84</v>
-      </c>
       <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
-        <v>4</v>
-      </c>
       <c r="K1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>19</v>
@@ -1059,22 +1008,22 @@
       <c r="G2" t="s">
         <v>0</v>
       </c>
-      <c r="H2" t="s">
-        <v>55</v>
+      <c r="H2" s="2">
+        <v>3</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>19</v>
@@ -1095,15 +1044,15 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1117,22 +1066,22 @@
       <c r="F4" t="s">
         <v>0</v>
       </c>
-      <c r="G4" t="s">
-        <v>56</v>
+      <c r="G4" s="2">
+        <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I4" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1146,8 +1095,8 @@
       <c r="F5" t="s">
         <v>0</v>
       </c>
-      <c r="G5" t="s">
-        <v>56</v>
+      <c r="G5" s="2">
+        <v>1</v>
       </c>
       <c r="H5" t="s">
         <v>0</v>
@@ -1155,10 +1104,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C6">
         <v>31</v>
@@ -1172,31 +1121,31 @@
       <c r="F6" t="s">
         <v>0</v>
       </c>
-      <c r="G6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H6" t="s">
-        <v>56</v>
+      <c r="G6" s="2">
+        <v>3</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
       </c>
       <c r="I6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" t="s">
         <v>16</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" t="s">
         <v>17</v>
-      </c>
-      <c r="K6" t="s">
-        <v>40</v>
-      </c>
-      <c r="L6" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C7">
         <v>51</v>
@@ -1205,27 +1154,27 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" t="s">
         <v>56</v>
       </c>
-      <c r="H7" t="s">
-        <v>56</v>
+      <c r="F7" s="2">
+        <v>4</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -1248,10 +1197,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C9">
         <v>12</v>
@@ -1268,28 +1217,28 @@
       <c r="G9" t="s">
         <v>0</v>
       </c>
-      <c r="H9" t="s">
-        <v>56</v>
+      <c r="H9" s="2">
+        <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L9" t="s">
         <v>30</v>
-      </c>
-      <c r="L9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C10">
         <v>4</v>
@@ -1312,10 +1261,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B11" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C11">
         <v>15</v>
@@ -1329,19 +1278,19 @@
       <c r="F11" t="s">
         <v>0</v>
       </c>
-      <c r="G11" t="s">
-        <v>2</v>
-      </c>
-      <c r="H11" t="s">
-        <v>55</v>
+      <c r="G11" s="2">
+        <v>7</v>
+      </c>
+      <c r="H11" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C12">
         <v>3</v>
@@ -1383,48 +1332,48 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>60</v>
@@ -1439,21 +1388,21 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>33</v>
@@ -1468,15 +1417,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>16</v>
@@ -1491,24 +1440,24 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
       <c r="I4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>20</v>
@@ -1517,30 +1466,30 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C6">
         <v>3</v>
@@ -1555,18 +1504,18 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C7">
         <v>12</v>
@@ -1601,42 +1550,42 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>55</v>
@@ -1651,18 +1600,18 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>13</v>
@@ -1671,21 +1620,21 @@
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>26</v>
@@ -1697,24 +1646,24 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>44</v>
@@ -1723,30 +1672,30 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C6">
         <v>10</v>
@@ -1763,10 +1712,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1781,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1805,42 +1754,42 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>55</v>
@@ -1855,15 +1804,15 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>13</v>
@@ -1878,15 +1827,15 @@
         <v>4</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>13</v>
@@ -1903,10 +1852,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>81</v>
@@ -1921,24 +1870,24 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
         <v>53</v>
       </c>
-      <c r="I5" t="s">
-        <v>54</v>
-      </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C6">
         <v>6</v>
@@ -1955,10 +1904,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C7">
         <v>16</v>
@@ -1973,13 +1922,13 @@
         <v>2</v>
       </c>
       <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
         <v>16</v>
       </c>
-      <c r="H7" t="s">
-        <v>17</v>
-      </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2002,42 +1951,42 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>36</v>
@@ -2052,15 +2001,15 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>9</v>
@@ -2075,15 +2024,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>14</v>
@@ -2100,10 +2049,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>27</v>
@@ -2118,18 +2067,18 @@
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C6">
         <v>80</v>
@@ -2144,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" t="s">
         <v>53</v>
       </c>
-      <c r="I6" t="s">
-        <v>54</v>
-      </c>
       <c r="J6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2181,72 +2130,72 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="T1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4">
         <f>SUM(C2:D2)</f>
@@ -2265,10 +2214,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E12" si="0">SUM(C3:D3)</f>
@@ -2287,10 +2236,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
@@ -2309,10 +2258,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>17</v>
@@ -2337,10 +2286,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>2</v>
@@ -2363,18 +2312,18 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4">
         <v>23</v>
@@ -2397,15 +2346,15 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C8" s="4">
         <v>0</v>
@@ -2430,10 +2379,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>7</v>
@@ -2458,10 +2407,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>12</v>
@@ -2486,10 +2435,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="4">
         <v>187</v>
@@ -2518,24 +2467,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>21</v>
@@ -2548,10 +2497,10 @@
         <v>21</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>114</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2580,72 +2529,72 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="T1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4">
         <f>SUM(C2:D2)</f>
@@ -2667,10 +2616,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E12" si="0">SUM(C3:D3)</f>
@@ -2692,10 +2641,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
@@ -2717,10 +2666,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>8</v>
@@ -2748,10 +2697,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>2</v>
@@ -2780,18 +2729,18 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -2817,15 +2766,15 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C8" s="4">
         <v>0</v>
@@ -2853,10 +2802,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
@@ -2884,10 +2833,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -2915,10 +2864,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="4">
         <v>84</v>
@@ -2950,24 +2899,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>17</v>
@@ -2989,13 +2938,13 @@
         <v>0</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>115</v>
+        <v>16</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>114</v>
+        <v>51</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3024,72 +2973,72 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="T1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4">
         <f>SUM(C2:D2)</f>
@@ -3111,10 +3060,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E11" si="0">SUM(C3:D3)</f>
@@ -3136,10 +3085,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
@@ -3161,10 +3110,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>8</v>
@@ -3189,10 +3138,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>3</v>
@@ -3221,18 +3170,18 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -3255,15 +3204,15 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C8" s="4">
         <v>0</v>
@@ -3288,10 +3237,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
@@ -3316,10 +3265,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -3344,10 +3293,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="4">
         <v>186</v>
@@ -3379,24 +3328,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>7</v>
@@ -3405,10 +3354,10 @@
         <v>1</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>114</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -3437,72 +3386,72 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="T1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4">
         <f>SUM(C2:D2)</f>
@@ -3519,10 +3468,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E12" si="0">SUM(C3:D3)</f>
@@ -3539,10 +3488,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
@@ -3559,10 +3508,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>14</v>
@@ -3594,10 +3543,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>2</v>
@@ -3624,18 +3573,18 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4">
         <v>13</v>
@@ -3667,10 +3616,10 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C8" s="4">
         <v>1</v>
@@ -3702,10 +3651,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
@@ -3737,10 +3686,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -3763,10 +3712,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="4">
         <v>64</v>
@@ -3793,21 +3742,21 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>41</v>
@@ -3820,10 +3769,10 @@
         <v>43</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>115</v>
+        <v>16</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3852,72 +3801,72 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="T1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4">
         <f>SUM(C2:D2)</f>
@@ -3937,10 +3886,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E12" si="0">SUM(C3:D3)</f>
@@ -3960,10 +3909,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
@@ -3983,10 +3932,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>21</v>
@@ -4018,10 +3967,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>5</v>
@@ -4054,18 +4003,18 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4">
         <v>4</v>
@@ -4097,10 +4046,10 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C8" s="4">
         <v>1</v>
@@ -4132,10 +4081,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>6</v>
@@ -4167,10 +4116,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>1</v>
@@ -4196,10 +4145,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="4">
         <v>95</v>
@@ -4232,24 +4181,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>9</v>
@@ -4262,10 +4211,10 @@
         <v>9</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>114</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -4292,105 +4241,105 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="G1" s="4" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>4</v>
-      </c>
       <c r="J1" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="M1" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="P1" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C5" s="4">
         <v>1</v>
       </c>
       <c r="E5" s="4">
-        <f t="shared" ref="E3:E12" si="0">SUM(C5:D5)</f>
+        <f t="shared" ref="E5:E12" si="0">SUM(C5:D5)</f>
         <v>1</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>141</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>2</v>
@@ -4403,31 +4352,31 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>140</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4">
         <v>9</v>
@@ -4436,19 +4385,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>144</v>
-      </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C10" s="4">
         <v>1</v>
@@ -4458,15 +4401,15 @@
         <v>1</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C11" s="6">
         <v>194</v>
@@ -4482,42 +4425,30 @@
         <v>30</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="N11" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="O11" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="P11" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q11" s="7" t="s">
-        <v>149</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C12" s="4">
         <v>16</v>
@@ -4526,14 +4457,14 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="H12" s="6" t="s">
-        <v>113</v>
+      <c r="H12" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>114</v>
+        <v>16</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -4568,57 +4499,57 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>82</v>
       </c>
-      <c r="G1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H1" t="s">
-        <v>84</v>
-      </c>
       <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
-        <v>4</v>
-      </c>
       <c r="K1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>71</v>
@@ -4639,33 +4570,33 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" t="s">
         <v>63</v>
       </c>
-      <c r="K2" t="s">
-        <v>35</v>
-      </c>
-      <c r="L2" t="s">
-        <v>64</v>
-      </c>
-      <c r="M2" t="s">
-        <v>65</v>
-      </c>
       <c r="N2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>24</v>
@@ -4686,23 +4617,23 @@
         <v>17</v>
       </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -4723,15 +4654,15 @@
         <v>2</v>
       </c>
       <c r="I5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C6">
         <v>32</v>
@@ -4754,10 +4685,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C7">
         <v>68</v>
@@ -4780,10 +4711,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="C8">
         <v>3</v>
@@ -4804,15 +4735,15 @@
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -4835,10 +4766,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C10">
         <v>14</v>
@@ -4861,10 +4792,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B11" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -4887,10 +4818,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C12">
         <v>15</v>
@@ -4913,10 +4844,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C13">
         <v>4</v>
@@ -4939,10 +4870,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -4963,7 +4894,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -4986,48 +4917,48 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>77</v>
@@ -5042,27 +4973,27 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>28</v>
@@ -5077,15 +5008,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -5100,15 +5031,15 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>23</v>
@@ -5123,27 +5054,27 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>16</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>18</v>
-      </c>
-      <c r="K5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C6">
         <v>29</v>
@@ -5152,24 +5083,24 @@
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -5184,15 +5115,15 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -5207,24 +5138,24 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8" t="s">
         <v>30</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9">
         <v>31</v>
@@ -5241,10 +5172,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -5261,10 +5192,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -5279,7 +5210,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -5309,48 +5240,48 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>62</v>
@@ -5365,30 +5296,30 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -5403,15 +5334,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -5426,15 +5357,15 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>32</v>
@@ -5449,24 +5380,24 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>16</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>18</v>
-      </c>
-      <c r="J5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C6">
         <v>32</v>
@@ -5481,18 +5412,18 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
         <v>20</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -5507,15 +5438,15 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -5530,18 +5461,18 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
         <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9">
         <v>22</v>
@@ -5581,48 +5512,48 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>74</v>
@@ -5637,24 +5568,24 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" t="s">
         <v>10</v>
-      </c>
-      <c r="J2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>24</v>
@@ -5669,15 +5600,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -5692,18 +5623,18 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
         <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>22</v>
@@ -5718,18 +5649,18 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C6">
         <v>32</v>
@@ -5744,24 +5675,24 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>28</v>
-      </c>
-      <c r="I6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -5778,10 +5709,10 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -5796,21 +5727,21 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" t="s">
         <v>30</v>
       </c>
-      <c r="H8" t="s">
-        <v>31</v>
-      </c>
       <c r="J8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9">
         <v>28</v>
@@ -5827,10 +5758,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -5847,10 +5778,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -5885,57 +5816,57 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" t="s">
         <v>36</v>
       </c>
-      <c r="N1" t="s">
-        <v>37</v>
-      </c>
       <c r="O1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>81</v>
@@ -5950,33 +5881,33 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
         <v>33</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>34</v>
       </c>
-      <c r="K2" t="s">
-        <v>35</v>
-      </c>
       <c r="L2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>22</v>
@@ -5991,15 +5922,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -6014,15 +5945,15 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C5">
         <v>16</v>
@@ -6037,24 +5968,24 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>16</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" t="s">
         <v>17</v>
-      </c>
-      <c r="I5" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C6">
         <v>63</v>
@@ -6063,33 +5994,33 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
       </c>
       <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" t="s">
-        <v>21</v>
-      </c>
       <c r="J6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -6104,15 +6035,15 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -6127,15 +6058,15 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C9">
         <v>28</v>
@@ -6152,10 +6083,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -6190,54 +6121,54 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" t="s">
         <v>36</v>
-      </c>
-      <c r="N1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>63</v>
@@ -6252,33 +6183,33 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" t="s">
         <v>34</v>
       </c>
-      <c r="I2" t="s">
-        <v>35</v>
-      </c>
       <c r="J2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -6293,15 +6224,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>14</v>
@@ -6316,18 +6247,18 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>34</v>
@@ -6336,30 +6267,30 @@
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
       </c>
       <c r="G5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" t="s">
         <v>20</v>
       </c>
-      <c r="H5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" t="s">
-        <v>21</v>
-      </c>
       <c r="J5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -6374,18 +6305,18 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C7">
         <v>14</v>
@@ -6402,10 +6333,10 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -6440,54 +6371,54 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" t="s">
         <v>36</v>
-      </c>
-      <c r="N1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>53</v>
@@ -6502,24 +6433,24 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>27</v>
@@ -6534,15 +6465,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>30</v>
@@ -6557,27 +6488,27 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
       <c r="I4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>29</v>
@@ -6592,21 +6523,21 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C6">
         <v>7</v>
@@ -6621,18 +6552,18 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C7">
         <v>13</v>
@@ -6667,42 +6598,42 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
-      <c r="E1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
       <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>42</v>
@@ -6717,18 +6648,18 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>32</v>
@@ -6743,15 +6674,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>32</v>
@@ -6766,18 +6697,18 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C5">
         <v>42</v>
@@ -6786,24 +6717,24 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -6820,10 +6751,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C7">
         <v>14</v>

</xml_diff>

<commit_message>
corrected an error in FY21 peer review data for HHS (total peer reviews were not calculated from ISI and HISA)
</commit_message>
<xml_diff>
--- a/bin/peer_review_source.xlsx
+++ b/bin/peer_review_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9457C3B5-DD71-42CA-A0E4-4208B86B6A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09E3686-E76B-49B6-A21C-FE676EB90636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="17" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="18" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
   </bookViews>
   <sheets>
     <sheet name="FY06" sheetId="15" r:id="rId1"/>
@@ -3066,7 +3066,7 @@
         <v>119</v>
       </c>
       <c r="E3" s="4">
-        <f t="shared" ref="E3:E11" si="0">SUM(C3:D3)</f>
+        <f t="shared" ref="E3:E12" si="0">SUM(C3:D3)</f>
         <v>0</v>
       </c>
       <c r="H3" s="4">
@@ -3352,6 +3352,10 @@
       </c>
       <c r="D12" s="4">
         <v>1</v>
+      </c>
+      <c r="E12" s="4">
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Corrected FY23 EPA peer review data; EPA found they had not submitted complete data for FY23 during the FY19-23 catch-up data call
</commit_message>
<xml_diff>
--- a/bin/peer_review_source.xlsx
+++ b/bin/peer_review_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09E3686-E76B-49B6-A21C-FE676EB90636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3F28E0-9055-4A70-AA2A-829AEEB17C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="18" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="17" xr2:uid="{7275623A-AD6D-410F-A905-5A05365876F9}"/>
   </bookViews>
   <sheets>
     <sheet name="FY06" sheetId="15" r:id="rId1"/>
@@ -4091,16 +4091,19 @@
         <v>114</v>
       </c>
       <c r="C9" s="4">
+        <v>9</v>
+      </c>
+      <c r="D9" s="4">
         <v>6</v>
-      </c>
-      <c r="D9" s="4">
-        <v>5</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
         <v>0</v>
       </c>
       <c r="H9" s="4">

</xml_diff>